<commit_message>
Update Gemini vs OpenAI Full Report with new data. The binary file `Gemini_vs_OpenAI_Full_Report_v2.xlsx` has been modified to reflect the latest API data and analysis.
</commit_message>
<xml_diff>
--- a/Gemini_vs_OpenAI_Full_Report_v2.xlsx
+++ b/Gemini_vs_OpenAI_Full_Report_v2.xlsx
@@ -1504,7 +1504,7 @@
       </c>
       <c r="CE3" s="23" t="inlineStr">
         <is>
-          <t>new_inquiry, warm, not_booked, Shingle replacement</t>
+          <t>not_booked, new_inquiry, warm, Shingle replacement</t>
         </is>
       </c>
     </row>
@@ -1890,7 +1890,7 @@
       </c>
       <c r="CE4" s="24" t="inlineStr">
         <is>
-          <t>new_inquiry, warm, Roof repair, booked</t>
+          <t>Roof repair, new_inquiry, warm, booked</t>
         </is>
       </c>
     </row>
@@ -2207,7 +2207,7 @@
       </c>
       <c r="CE5" s="23" t="inlineStr">
         <is>
-          <t>roof tile replacement, hot, service_not_offered, new_inquiry</t>
+          <t>new_inquiry, service_not_offered, roof tile replacement, hot</t>
         </is>
       </c>
     </row>
@@ -2556,7 +2556,7 @@
       </c>
       <c r="CE6" s="24" t="inlineStr">
         <is>
-          <t>roof repair, new_inquiry, warm, not_booked</t>
+          <t>not_booked, roof repair, new_inquiry, warm</t>
         </is>
       </c>
     </row>
@@ -2862,7 +2862,7 @@
       </c>
       <c r="CE7" s="23" t="inlineStr">
         <is>
-          <t>quote_only, warm, Tiled roof, not_booked</t>
+          <t>not_booked, Tiled roof, warm, quote_only</t>
         </is>
       </c>
     </row>
@@ -3227,7 +3227,7 @@
       </c>
       <c r="CE8" s="24" t="inlineStr">
         <is>
-          <t>new_inquiry, Roof inspection, warm, not_booked</t>
+          <t>not_booked, new_inquiry, warm, Roof inspection</t>
         </is>
       </c>
     </row>
@@ -3577,7 +3577,7 @@
       </c>
       <c r="CE9" s="23" t="inlineStr">
         <is>
-          <t>new_inquiry, service_not_offered, warm, Roof and skylight inspection and estimate</t>
+          <t>Roof and skylight inspection and estimate, new_inquiry, warm, service_not_offered</t>
         </is>
       </c>
     </row>
@@ -3921,7 +3921,7 @@
       </c>
       <c r="CE10" s="24" t="inlineStr">
         <is>
-          <t>new_inquiry, cold, Porch roof repair, not_booked</t>
+          <t>cold, not_booked, Porch roof repair, new_inquiry</t>
         </is>
       </c>
     </row>
@@ -4263,7 +4263,7 @@
       </c>
       <c r="CE11" s="23" t="inlineStr">
         <is>
-          <t>Roof inspection follow-up, cold, follow_up, not_booked</t>
+          <t>cold, not_booked, Roof inspection follow-up, follow_up</t>
         </is>
       </c>
     </row>
@@ -4646,7 +4646,7 @@
       </c>
       <c r="CE12" s="24" t="inlineStr">
         <is>
-          <t>warm, confirmation, not_booked</t>
+          <t>not_booked, warm, confirmation</t>
         </is>
       </c>
     </row>
@@ -4916,7 +4916,7 @@
       </c>
       <c r="CE13" s="23" t="inlineStr">
         <is>
-          <t>follow_up, not_booked, unqualified</t>
+          <t>not_booked, follow_up, unqualified</t>
         </is>
       </c>
     </row>
@@ -5286,7 +5286,7 @@
       </c>
       <c r="CE14" s="24" t="inlineStr">
         <is>
-          <t>new_inquiry, cold, not_booked, Roof replacement</t>
+          <t>cold, not_booked, Roof replacement, new_inquiry</t>
         </is>
       </c>
     </row>
@@ -5660,7 +5660,7 @@
       </c>
       <c r="CE15" s="23" t="inlineStr">
         <is>
-          <t>new_inquiry, cold, not_booked, Roof inspection</t>
+          <t>cold, not_booked, new_inquiry, Roof inspection</t>
         </is>
       </c>
     </row>
@@ -6045,7 +6045,7 @@
       </c>
       <c r="CE16" s="24" t="inlineStr">
         <is>
-          <t>new_inquiry, Roof inspection, warm, booked</t>
+          <t>Roof inspection, new_inquiry, warm, booked</t>
         </is>
       </c>
     </row>
@@ -6487,7 +6487,7 @@
       </c>
       <c r="CE18" s="24" t="inlineStr">
         <is>
-          <t>Roof repair estimate, warm, follow_up, booked</t>
+          <t>follow_up, Roof repair estimate, warm, booked</t>
         </is>
       </c>
     </row>
@@ -6753,7 +6753,7 @@
       </c>
       <c r="CE19" s="23" t="inlineStr">
         <is>
-          <t>booked, follow_up, unqualified</t>
+          <t>follow_up, unqualified, booked</t>
         </is>
       </c>
     </row>
@@ -7145,7 +7145,7 @@
       </c>
       <c r="CE20" s="24" t="inlineStr">
         <is>
-          <t>hot, new_inquiry, booked, Roof repair and replacement estimate</t>
+          <t>Roof repair and replacement estimate, new_inquiry, booked, hot</t>
         </is>
       </c>
     </row>
@@ -7482,7 +7482,7 @@
       </c>
       <c r="CE21" s="23" t="inlineStr">
         <is>
-          <t>new_inquiry, cold, Replace clay tile patio roofs with metal, not_booked</t>
+          <t>cold, not_booked, Replace clay tile patio roofs with metal, new_inquiry</t>
         </is>
       </c>
     </row>
@@ -7873,7 +7873,7 @@
       </c>
       <c r="CE22" s="24" t="inlineStr">
         <is>
-          <t>hot, new_inquiry, booked, Roof inspection and estimate for leaking roof</t>
+          <t>Roof inspection and estimate for leaking roof, new_inquiry, booked, hot</t>
         </is>
       </c>
     </row>
@@ -8216,7 +8216,7 @@
       </c>
       <c r="CE23" s="23" t="inlineStr">
         <is>
-          <t>warm, confirmation, not_booked</t>
+          <t>not_booked, warm, confirmation</t>
         </is>
       </c>
     </row>
@@ -8600,7 +8600,7 @@
       </c>
       <c r="CE24" s="24" t="inlineStr">
         <is>
-          <t>hot, new_inquiry, booked, Roof inspection and replacement estimate for leak</t>
+          <t>new_inquiry, Roof inspection and replacement estimate for leak, booked, hot</t>
         </is>
       </c>
     </row>
@@ -8875,7 +8875,7 @@
       </c>
       <c r="CE25" s="23" t="inlineStr">
         <is>
-          <t>new_inquiry, not_booked, unqualified</t>
+          <t>not_booked, unqualified, new_inquiry</t>
         </is>
       </c>
     </row>
@@ -9224,7 +9224,7 @@
       </c>
       <c r="CE26" s="24" t="inlineStr">
         <is>
-          <t>new_inquiry, warm, not_booked, Roof repair quote</t>
+          <t>not_booked, Roof repair quote, new_inquiry, warm</t>
         </is>
       </c>
     </row>
@@ -9496,7 +9496,7 @@
       </c>
       <c r="CE27" s="23" t="inlineStr">
         <is>
-          <t>confirmation, not_booked, unqualified</t>
+          <t>not_booked, unqualified, confirmation</t>
         </is>
       </c>
     </row>
@@ -9768,7 +9768,7 @@
       </c>
       <c r="CE28" s="24" t="inlineStr">
         <is>
-          <t>new_inquiry, not_booked, unqualified</t>
+          <t>not_booked, unqualified, new_inquiry</t>
         </is>
       </c>
     </row>
@@ -10037,7 +10037,7 @@
       </c>
       <c r="CE29" s="23" t="inlineStr">
         <is>
-          <t>follow_up, not_booked, unqualified</t>
+          <t>not_booked, follow_up, unqualified</t>
         </is>
       </c>
     </row>
@@ -10309,7 +10309,7 @@
       </c>
       <c r="CE30" s="24" t="inlineStr">
         <is>
-          <t>follow_up, not_booked, unqualified</t>
+          <t>not_booked, follow_up, unqualified</t>
         </is>
       </c>
     </row>
@@ -10617,7 +10617,7 @@
       </c>
       <c r="CE31" s="23" t="inlineStr">
         <is>
-          <t>follow_up, not_booked, unqualified</t>
+          <t>not_booked, follow_up, unqualified</t>
         </is>
       </c>
     </row>
@@ -10939,7 +10939,7 @@
       </c>
       <c r="CE32" s="24" t="inlineStr">
         <is>
-          <t>hot, new_inquiry, not_booked, Roof repair estimate</t>
+          <t>not_booked, new_inquiry, Roof repair estimate, hot</t>
         </is>
       </c>
     </row>
@@ -11861,7 +11861,7 @@
       </c>
       <c r="CE3" s="23" t="inlineStr">
         <is>
-          <t>new_inquiry, warm, not_booked, Roofing estimate/quote for shingle replacement</t>
+          <t>not_booked, new_inquiry, warm, Roofing estimate/quote for shingle replacement</t>
         </is>
       </c>
     </row>
@@ -12238,7 +12238,7 @@
       </c>
       <c r="CE4" s="24" t="inlineStr">
         <is>
-          <t>hot, new_inquiry, Roof repair (replace/fix fallen roof tiles; no active leak), not_booked</t>
+          <t>not_booked, new_inquiry, Roof repair (replace/fix fallen roof tiles; no active leak), hot</t>
         </is>
       </c>
     </row>
@@ -12523,7 +12523,7 @@
       </c>
       <c r="CE5" s="23" t="inlineStr">
         <is>
-          <t>new_inquiry, not_booked, unqualified</t>
+          <t>not_booked, unqualified, new_inquiry</t>
         </is>
       </c>
     </row>
@@ -12880,7 +12880,7 @@
       </c>
       <c r="CE6" s="24" t="inlineStr">
         <is>
-          <t>warm, confirmation, not_booked, Commercial roof repair</t>
+          <t>not_booked, Commercial roof repair, warm, confirmation</t>
         </is>
       </c>
     </row>
@@ -13203,7 +13203,7 @@
       </c>
       <c r="CE7" s="23" t="inlineStr">
         <is>
-          <t>quote_only, warm, not_booked, Tiled roof pricing/estimate inquiry</t>
+          <t>not_booked, Tiled roof pricing/estimate inquiry, warm, quote_only</t>
         </is>
       </c>
     </row>
@@ -13573,7 +13573,7 @@
       </c>
       <c r="CE8" s="24" t="inlineStr">
         <is>
-          <t>new_inquiry, Roof inspection, warm, not_booked</t>
+          <t>not_booked, new_inquiry, warm, Roof inspection</t>
         </is>
       </c>
     </row>
@@ -14029,7 +14029,7 @@
       </c>
       <c r="CE10" s="24" t="inlineStr">
         <is>
-          <t>new_inquiry, warm, not_booked, Porch roof repair/estimate (possible fascia/plywood/boarding replacement under tile; potential structural wood repair)</t>
+          <t>not_booked, new_inquiry, warm, Porch roof repair/estimate (possible fascia/plywood/boarding replacement under tile; potential structural wood repair)</t>
         </is>
       </c>
     </row>
@@ -14383,7 +14383,7 @@
       </c>
       <c r="CE11" s="23" t="inlineStr">
         <is>
-          <t>warm, Roof inspection (status follow-up from prior inspection), follow_up, booked</t>
+          <t>follow_up, Roof inspection (status follow-up from prior inspection), warm, booked</t>
         </is>
       </c>
     </row>
@@ -14766,7 +14766,7 @@
       </c>
       <c r="CE12" s="24" t="inlineStr">
         <is>
-          <t>warm, confirmation, not_booked</t>
+          <t>not_booked, warm, confirmation</t>
         </is>
       </c>
     </row>
@@ -15047,7 +15047,7 @@
       </c>
       <c r="CE13" s="23" t="inlineStr">
         <is>
-          <t>booked, follow_up, unqualified</t>
+          <t>follow_up, unqualified, booked</t>
         </is>
       </c>
     </row>
@@ -15426,7 +15426,7 @@
       </c>
       <c r="CE14" s="24" t="inlineStr">
         <is>
-          <t>new_inquiry, cold, Roof replacement quote, not_booked</t>
+          <t>cold, not_booked, Roof replacement quote, new_inquiry</t>
         </is>
       </c>
     </row>
@@ -15797,7 +15797,7 @@
       </c>
       <c r="CE15" s="23" t="inlineStr">
         <is>
-          <t>new_inquiry, cold, not_booked, Roof inspection for real estate sale/insurance-damage assessment with written report and options</t>
+          <t>cold, not_booked, new_inquiry, Roof inspection for real estate sale/insurance-damage assessment with written report and options</t>
         </is>
       </c>
     </row>
@@ -16622,7 +16622,7 @@
       </c>
       <c r="CE17" s="23" t="inlineStr">
         <is>
-          <t>hot, new_inquiry, booked, Free roof inspection and quote for roof repairs (leaks/ceiling collapse concerns) on tile roof</t>
+          <t>Free roof inspection and quote for roof repairs (leaks/ceiling collapse concerns) on tile roof, new_inquiry, booked, hot</t>
         </is>
       </c>
     </row>
@@ -16981,7 +16981,7 @@
       </c>
       <c r="CE18" s="24" t="inlineStr">
         <is>
-          <t>warm, follow_up, booked, Roof repair estimate / roof repair</t>
+          <t>Roof repair estimate / roof repair, follow_up, warm, booked</t>
         </is>
       </c>
     </row>
@@ -17255,7 +17255,7 @@
       </c>
       <c r="CE19" s="23" t="inlineStr">
         <is>
-          <t>booked, follow_up, unqualified</t>
+          <t>follow_up, unqualified, booked</t>
         </is>
       </c>
     </row>
@@ -17655,7 +17655,7 @@
       </c>
       <c r="CE20" s="24" t="inlineStr">
         <is>
-          <t>Roof inspection and estimate for wind/rain damage repairs and potential full roof replacement (asphalt shingles vs metal roof option) on a manufactured home including porch roof areas, hot, new_inquiry, booked</t>
+          <t>Roof inspection and estimate for wind/rain damage repairs and potential full roof replacement (asphalt shingles vs metal roof option) on a manufactured home including porch roof areas, new_inquiry, booked, hot</t>
         </is>
       </c>
     </row>
@@ -17992,7 +17992,7 @@
       </c>
       <c r="CE21" s="23" t="inlineStr">
         <is>
-          <t>Roof replacement (replace clay tile patio roofs with metal), new_inquiry, cold, not_booked</t>
+          <t>cold, not_booked, Roof replacement (replace clay tile patio roofs with metal), new_inquiry</t>
         </is>
       </c>
     </row>
@@ -18369,7 +18369,7 @@
       </c>
       <c r="CE22" s="24" t="inlineStr">
         <is>
-          <t>new_inquiry, Free comprehensive roof inspection and estimate for a leaking garage tile roof, warm, booked</t>
+          <t>Free comprehensive roof inspection and estimate for a leaking garage tile roof, new_inquiry, warm, booked</t>
         </is>
       </c>
     </row>
@@ -18646,7 +18646,7 @@
       </c>
       <c r="CE23" s="23" t="inlineStr">
         <is>
-          <t>confirmation, not_booked, unqualified</t>
+          <t>not_booked, unqualified, confirmation</t>
         </is>
       </c>
     </row>
@@ -19013,7 +19013,7 @@
       </c>
       <c r="CE24" s="24" t="inlineStr">
         <is>
-          <t>hot, new_inquiry, booked, Roof inspection/estimate for leaking shingle roof (possible repair or replacement)</t>
+          <t>Roof inspection/estimate for leaking shingle roof (possible repair or replacement), new_inquiry, booked, hot</t>
         </is>
       </c>
     </row>
@@ -19288,7 +19288,7 @@
       </c>
       <c r="CE25" s="23" t="inlineStr">
         <is>
-          <t>follow_up, not_booked, unqualified</t>
+          <t>not_booked, follow_up, unqualified</t>
         </is>
       </c>
     </row>
@@ -19658,7 +19658,7 @@
       </c>
       <c r="CE26" s="24" t="inlineStr">
         <is>
-          <t>new_inquiry, warm, not_booked, Roof inspection and estimate/quote for repairs or replacement (real estate transaction roof report)</t>
+          <t>not_booked, Roof inspection and estimate/quote for repairs or replacement (real estate transaction roof report), new_inquiry, warm</t>
         </is>
       </c>
     </row>
@@ -19933,7 +19933,7 @@
       </c>
       <c r="CE27" s="23" t="inlineStr">
         <is>
-          <t>follow_up, not_booked, unqualified</t>
+          <t>not_booked, follow_up, unqualified</t>
         </is>
       </c>
     </row>
@@ -20207,7 +20207,7 @@
       </c>
       <c r="CE28" s="24" t="inlineStr">
         <is>
-          <t>follow_up, not_booked, unqualified</t>
+          <t>not_booked, follow_up, unqualified</t>
         </is>
       </c>
     </row>
@@ -20515,7 +20515,7 @@
       </c>
       <c r="CE29" s="23" t="inlineStr">
         <is>
-          <t>booked, follow_up, unqualified</t>
+          <t>follow_up, unqualified, booked</t>
         </is>
       </c>
     </row>
@@ -20793,7 +20793,7 @@
       </c>
       <c r="CE30" s="24" t="inlineStr">
         <is>
-          <t>follow_up, not_booked, unqualified</t>
+          <t>not_booked, follow_up, unqualified</t>
         </is>
       </c>
     </row>
@@ -21105,7 +21105,7 @@
       </c>
       <c r="CE31" s="23" t="inlineStr">
         <is>
-          <t>follow_up, not_booked, unqualified</t>
+          <t>not_booked, follow_up, unqualified</t>
         </is>
       </c>
     </row>
@@ -21439,7 +21439,7 @@
       </c>
       <c r="CE32" s="24" t="inlineStr">
         <is>
-          <t>new_inquiry, warm, not_booked, Roof repair estimate and inspection</t>
+          <t>not_booked, Roof repair estimate and inspection, new_inquiry, warm</t>
         </is>
       </c>
     </row>

</xml_diff>